<commit_message>
The C Q3.2026: viet lai Truoc cai tien va tieu de, them bang so sanh, giu anh file doi chieu, thiet lap in 1 trang A4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D813CqnTusevYBx6CZme3b
</commit_message>
<xml_diff>
--- a/The C cai tien/De an cai tien Q3.2026_ban sua.xlsx
+++ b/The C cai tien/De an cai tien Q3.2026_ban sua.xlsx
@@ -8,7 +8,9 @@
   <sheets>
     <sheet name="Nội dung" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Nội dung'!$A$2:$AG$49</definedName>
+  </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="20">
     <font>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
@@ -89,17 +91,47 @@
     </font>
     <font>
       <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Times New Roman"/>
-      <color rgb="FF3C4043"/>
-      <sz val="11"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -110,7 +142,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="61">
+  <borders count="73">
     <border>
       <left/>
       <right/>
@@ -847,6 +879,78 @@
         <color indexed="64"/>
       </bottom>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="3">
@@ -854,7 +958,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1242,31 +1346,64 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="61" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="70" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="70" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1343,6 +1480,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>17</col>
+      <colOff>173935</colOff>
+      <row>17</row>
+      <rowOff>15000</rowOff>
+    </from>
+    <ext cx="6168622" cy="1651886"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1644,7 +1811,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:AJ49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
@@ -2287,8 +2454,39 @@
       <c r="F5" s="134" t="n"/>
       <c r="G5" s="135" t="inlineStr">
         <is>
-          <t>Tự động hóa đối chiếu PO hàng tuần giữa Mua hàng và Kế hoạch lắp ráp (Power Query)
-購買課・計画課間のPO週次クロスチェック自動化【Power Query活用】</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <b val="1"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Hướng tới "0 PO bị sót": Tự động đối chiếu Yêu cầu mua ⇔ PO hàng tuần
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">(Mua hàng × Kế hoạch lắp ráp – ứng dụng Power Query)
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <b val="1"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">「発注漏れゼロ」へ：購入依頼⇔PO 週次自動照合
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <sz val="11"/>
+            </rPr>
+            <t>（購買課×組立計画課、Power Query活用）</t>
+          </r>
         </is>
       </c>
       <c r="U5" s="136" t="n"/>
@@ -2413,10 +2611,10 @@
       <c r="AF8" s="6" t="n"/>
       <c r="AG8" s="8" t="n"/>
     </row>
-    <row r="9" ht="16.95" customHeight="1">
+    <row r="9" ht="19" customHeight="1">
       <c r="A9" s="148" t="inlineStr">
         <is>
-          <t>Mua hàng chỉ đối chiếu hàng về với kho (ngày hôm sau), chưa có cơ chế đối chiếu</t>
+          <t>Đơn đã đặt thì có kiểm tra – đơn bị sót thì không ai nhìn thấy.</t>
         </is>
       </c>
       <c r="B9" s="11" t="n"/>
@@ -2437,7 +2635,7 @@
       <c r="Q9" s="16" t="n"/>
       <c r="R9" s="149" t="inlineStr">
         <is>
-          <t>Hợp nhất dữ liệu Mua hàng và Kế hoạch thành 1 file chung bằng Power Query</t>
+          <t>Đưa điểm kiểm tra lên đầu nguồn: đối chiếu Yêu cầu mua ⇔ PO tự động mỗi tuần.</t>
         </is>
       </c>
       <c r="S9" s="11" t="n"/>
@@ -2456,10 +2654,10 @@
       <c r="AF9" s="11" t="n"/>
       <c r="AG9" s="13" t="n"/>
     </row>
-    <row r="10" ht="16.95" customHeight="1">
+    <row r="10" ht="19" customHeight="1">
       <c r="A10" s="148" t="inlineStr">
         <is>
-          <t>định kỳ với bộ phận yêu cầu mua (Kế hoạch lắp ráp).</t>
+          <t>発注したPOは確認されるが、発注漏れは誰にも見えない。</t>
         </is>
       </c>
       <c r="B10" s="11" t="n"/>
@@ -2480,7 +2678,7 @@
       <c r="Q10" s="11" t="n"/>
       <c r="R10" s="150" t="inlineStr">
         <is>
-          <t>→ chỉ cần Refresh là tự động xuất danh sách chênh lệch.</t>
+          <t>チェックを上流へ：購入依頼とPOを毎週自動照合。</t>
         </is>
       </c>
       <c r="S10" s="11" t="n"/>
@@ -2499,12 +2697,8 @@
       <c r="AF10" s="11" t="n"/>
       <c r="AG10" s="13" t="n"/>
     </row>
-    <row r="11" ht="16.95" customHeight="1">
-      <c r="A11" s="151" t="inlineStr">
-        <is>
-          <t>→ Rủi ro sót / phát hành PO trễ, chỉ phát hiện khi đã ảnh hưởng sản xuất.</t>
-        </is>
-      </c>
+    <row r="11" ht="4" customHeight="1">
+      <c r="A11" s="48" t="n"/>
       <c r="B11" s="11" t="n"/>
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="11" t="n"/>
@@ -2521,11 +2715,7 @@
       <c r="O11" s="11" t="n"/>
       <c r="P11" s="11" t="n"/>
       <c r="Q11" s="11" t="n"/>
-      <c r="R11" s="150" t="inlineStr">
-        <is>
-          <t>→ 100% PO được đối chiếu hàng tuần, phát hiện sai lệch ngay trong tuần.</t>
-        </is>
-      </c>
+      <c r="R11" s="14" t="n"/>
       <c r="S11" s="11" t="n"/>
       <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
@@ -2542,137 +2732,183 @@
       <c r="AF11" s="11" t="n"/>
       <c r="AG11" s="13" t="n"/>
     </row>
-    <row r="12" ht="16.95" customHeight="1">
-      <c r="A12" s="148" t="inlineStr">
-        <is>
-          <t>購買は翌日に倉庫の入荷実績を確認しているが、発注依頼部署</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="11" t="n"/>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="151" t="inlineStr">
+        <is>
+          <t>Kế hoạch lắp ráp
+組立計画
+Yêu cầu mua / 購入依頼</t>
+        </is>
+      </c>
+      <c r="C12" s="152" t="n"/>
+      <c r="D12" s="153" t="n"/>
+      <c r="E12" s="154" t="inlineStr">
+        <is>
+          <t>Không đối chiếu</t>
+        </is>
+      </c>
+      <c r="G12" s="151" t="inlineStr">
+        <is>
+          <t>Mua hàng
+購買
+Phát hành PO / PO発行</t>
+        </is>
+      </c>
+      <c r="H12" s="152" t="n"/>
+      <c r="I12" s="152" t="n"/>
+      <c r="J12" s="152" t="n"/>
+      <c r="K12" s="153" t="n"/>
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="11" t="n"/>
-      <c r="N12" s="11" t="n"/>
-      <c r="O12" s="11" t="n"/>
-      <c r="P12" s="11" t="n"/>
-      <c r="Q12" s="11" t="n"/>
-      <c r="R12" s="152" t="inlineStr">
-        <is>
-          <t>購買データと計画データをPower Queryで一つの共通ファイルに統合し、</t>
-        </is>
-      </c>
-      <c r="S12" s="11" t="n"/>
-      <c r="T12" s="11" t="n"/>
-      <c r="U12" s="11" t="n"/>
-      <c r="V12" s="11" t="n"/>
-      <c r="W12" s="11" t="n"/>
-      <c r="X12" s="11" t="n"/>
-      <c r="Y12" s="11" t="n"/>
-      <c r="Z12" s="11" t="n"/>
-      <c r="AA12" s="11" t="n"/>
-      <c r="AB12" s="11" t="n"/>
-      <c r="AC12" s="11" t="n"/>
-      <c r="AD12" s="11" t="n"/>
-      <c r="AE12" s="11" t="n"/>
-      <c r="AF12" s="11" t="n"/>
+      <c r="N12" s="151" t="inlineStr">
+        <is>
+          <t>Hàng về kho / 入荷
+○ Check ngày hôm sau
+翌日実績チェック</t>
+        </is>
+      </c>
+      <c r="O12" s="152" t="n"/>
+      <c r="P12" s="152" t="n"/>
+      <c r="Q12" s="153" t="n"/>
+      <c r="R12" s="12" t="n"/>
+      <c r="S12" s="155" t="inlineStr">
+        <is>
+          <t>Hạng mục / 項目</t>
+        </is>
+      </c>
+      <c r="T12" s="156" t="n"/>
+      <c r="U12" s="156" t="n"/>
+      <c r="V12" s="157" t="n"/>
+      <c r="W12" s="155" t="inlineStr">
+        <is>
+          <t>Trước / 改善前</t>
+        </is>
+      </c>
+      <c r="X12" s="156" t="n"/>
+      <c r="Y12" s="156" t="n"/>
+      <c r="Z12" s="157" t="n"/>
+      <c r="AA12" s="155" t="inlineStr">
+        <is>
+          <t>Sau / 改善後</t>
+        </is>
+      </c>
+      <c r="AB12" s="156" t="n"/>
+      <c r="AC12" s="156" t="n"/>
+      <c r="AD12" s="156" t="n"/>
+      <c r="AE12" s="156" t="n"/>
+      <c r="AF12" s="157" t="n"/>
       <c r="AG12" s="13" t="n"/>
     </row>
-    <row r="13" ht="16.95" customHeight="1">
-      <c r="A13" s="148" t="inlineStr">
-        <is>
-          <t>（組立計画）との定期的な照合の仕組みがない。</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="11" t="n"/>
-      <c r="M13" s="11" t="n"/>
-      <c r="N13" s="11" t="n"/>
-      <c r="O13" s="11" t="n"/>
-      <c r="P13" s="11" t="n"/>
-      <c r="Q13" s="11" t="n"/>
-      <c r="R13" s="152" t="inlineStr">
-        <is>
-          <t>更新（Refresh）するだけで差異リストを自動抽出できる仕組みを構築。</t>
-        </is>
-      </c>
-      <c r="S13" s="11" t="n"/>
-      <c r="T13" s="11" t="n"/>
-      <c r="U13" s="11" t="n"/>
-      <c r="V13" s="11" t="n"/>
-      <c r="W13" s="11" t="n"/>
-      <c r="X13" s="11" t="n"/>
-      <c r="Y13" s="11" t="n"/>
-      <c r="Z13" s="11" t="n"/>
-      <c r="AA13" s="11" t="n"/>
-      <c r="AB13" s="11" t="n"/>
-      <c r="AC13" s="11" t="n"/>
-      <c r="AD13" s="11" t="n"/>
-      <c r="AE13" s="11" t="n"/>
-      <c r="AF13" s="11" t="n"/>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="158" t="n"/>
+      <c r="C13" s="159" t="n"/>
+      <c r="D13" s="160" t="n"/>
+      <c r="E13" s="161" t="inlineStr">
+        <is>
+          <t>✕ ――→</t>
+        </is>
+      </c>
+      <c r="G13" s="158" t="n"/>
+      <c r="H13" s="159" t="n"/>
+      <c r="I13" s="159" t="n"/>
+      <c r="J13" s="159" t="n"/>
+      <c r="K13" s="160" t="n"/>
+      <c r="L13" s="162" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="N13" s="158" t="n"/>
+      <c r="O13" s="159" t="n"/>
+      <c r="P13" s="159" t="n"/>
+      <c r="Q13" s="160" t="n"/>
+      <c r="R13" s="12" t="n"/>
+      <c r="S13" s="163" t="inlineStr">
+        <is>
+          <t>Tần suất / 照合頻度</t>
+        </is>
+      </c>
+      <c r="T13" s="156" t="n"/>
+      <c r="U13" s="156" t="n"/>
+      <c r="V13" s="157" t="n"/>
+      <c r="W13" s="163" t="inlineStr">
+        <is>
+          <t>Không định kỳ / 不定期</t>
+        </is>
+      </c>
+      <c r="X13" s="156" t="n"/>
+      <c r="Y13" s="156" t="n"/>
+      <c r="Z13" s="157" t="n"/>
+      <c r="AA13" s="155" t="inlineStr">
+        <is>
+          <t>1 lần/tuần / 週1回（定期）</t>
+        </is>
+      </c>
+      <c r="AB13" s="156" t="n"/>
+      <c r="AC13" s="156" t="n"/>
+      <c r="AD13" s="156" t="n"/>
+      <c r="AE13" s="156" t="n"/>
+      <c r="AF13" s="157" t="n"/>
       <c r="AG13" s="13" t="n"/>
     </row>
-    <row r="14" ht="16.95" customHeight="1">
-      <c r="A14" s="148" t="inlineStr">
-        <is>
-          <t>→PO漏れ・発行遅れのリスクがあり、生産に影響が出てから気づく。</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="164" t="n"/>
+      <c r="C14" s="165" t="n"/>
+      <c r="D14" s="166" t="n"/>
+      <c r="E14" s="154" t="inlineStr">
+        <is>
+          <t>照合なし</t>
+        </is>
+      </c>
+      <c r="G14" s="164" t="n"/>
+      <c r="H14" s="165" t="n"/>
+      <c r="I14" s="165" t="n"/>
+      <c r="J14" s="165" t="n"/>
+      <c r="K14" s="166" t="n"/>
       <c r="L14" s="11" t="n"/>
       <c r="M14" s="11" t="n"/>
-      <c r="N14" s="11" t="n"/>
-      <c r="O14" s="11" t="n"/>
-      <c r="P14" s="11" t="n"/>
-      <c r="Q14" s="11" t="n"/>
-      <c r="R14" s="152" t="inlineStr">
-        <is>
-          <t>→全POを毎週照合し、差異を週内に早期発見できる。</t>
-        </is>
-      </c>
-      <c r="S14" s="11" t="n"/>
-      <c r="T14" s="11" t="n"/>
-      <c r="U14" s="11" t="n"/>
-      <c r="V14" s="11" t="n"/>
-      <c r="W14" s="11" t="n"/>
-      <c r="X14" s="11" t="n"/>
-      <c r="Y14" s="11" t="n"/>
-      <c r="Z14" s="11" t="n"/>
-      <c r="AA14" s="11" t="n"/>
-      <c r="AB14" s="11" t="n"/>
-      <c r="AC14" s="11" t="n"/>
-      <c r="AD14" s="11" t="n"/>
-      <c r="AE14" s="11" t="n"/>
-      <c r="AF14" s="11" t="n"/>
+      <c r="N14" s="164" t="n"/>
+      <c r="O14" s="165" t="n"/>
+      <c r="P14" s="165" t="n"/>
+      <c r="Q14" s="166" t="n"/>
+      <c r="R14" s="12" t="n"/>
+      <c r="S14" s="163" t="inlineStr">
+        <is>
+          <t>Phương thức / 方法</t>
+        </is>
+      </c>
+      <c r="T14" s="156" t="n"/>
+      <c r="U14" s="156" t="n"/>
+      <c r="V14" s="157" t="n"/>
+      <c r="W14" s="163" t="inlineStr">
+        <is>
+          <t>Thủ công, Excel / 手作業</t>
+        </is>
+      </c>
+      <c r="X14" s="156" t="n"/>
+      <c r="Y14" s="156" t="n"/>
+      <c r="Z14" s="157" t="n"/>
+      <c r="AA14" s="155" t="inlineStr">
+        <is>
+          <t>Tự động, chỉ cần Refresh / 自動</t>
+        </is>
+      </c>
+      <c r="AB14" s="156" t="n"/>
+      <c r="AC14" s="156" t="n"/>
+      <c r="AD14" s="156" t="n"/>
+      <c r="AE14" s="156" t="n"/>
+      <c r="AF14" s="157" t="n"/>
       <c r="AG14" s="13" t="n"/>
     </row>
-    <row r="15" ht="16.95" customHeight="1">
-      <c r="A15" s="10" t="n"/>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="167" t="inlineStr">
+        <is>
+          <t>▲ Kiểm tra chỉ đặt ở cuối chuỗi (hàng về) → chỉ thấy đơn ĐÃ đặt.</t>
+        </is>
+      </c>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="11" t="n"/>
       <c r="D15" s="11" t="n"/>
@@ -2690,24 +2926,40 @@
       <c r="P15" s="11" t="n"/>
       <c r="Q15" s="11" t="n"/>
       <c r="R15" s="12" t="n"/>
-      <c r="S15" s="11" t="n"/>
-      <c r="T15" s="11" t="n"/>
-      <c r="U15" s="11" t="n"/>
-      <c r="V15" s="11" t="n"/>
-      <c r="W15" s="11" t="n"/>
-      <c r="X15" s="11" t="n"/>
-      <c r="Y15" s="11" t="n"/>
-      <c r="Z15" s="11" t="n"/>
-      <c r="AA15" s="11" t="n"/>
-      <c r="AB15" s="11" t="n"/>
-      <c r="AC15" s="11" t="n"/>
-      <c r="AD15" s="11" t="n"/>
-      <c r="AE15" s="11" t="n"/>
-      <c r="AF15" s="11" t="n"/>
+      <c r="S15" s="163" t="inlineStr">
+        <is>
+          <t>Phạm vi / 範囲</t>
+        </is>
+      </c>
+      <c r="T15" s="156" t="n"/>
+      <c r="U15" s="156" t="n"/>
+      <c r="V15" s="157" t="n"/>
+      <c r="W15" s="163" t="inlineStr">
+        <is>
+          <t>Chỉ đơn đã đặt / 発注済のみ</t>
+        </is>
+      </c>
+      <c r="X15" s="156" t="n"/>
+      <c r="Y15" s="156" t="n"/>
+      <c r="Z15" s="157" t="n"/>
+      <c r="AA15" s="155" t="inlineStr">
+        <is>
+          <t>100% yêu cầu mua / 全購入依頼</t>
+        </is>
+      </c>
+      <c r="AB15" s="156" t="n"/>
+      <c r="AC15" s="156" t="n"/>
+      <c r="AD15" s="156" t="n"/>
+      <c r="AE15" s="156" t="n"/>
+      <c r="AF15" s="157" t="n"/>
       <c r="AG15" s="13" t="n"/>
     </row>
-    <row r="16" ht="16.95" customHeight="1">
-      <c r="A16" s="10" t="n"/>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　 Đơn bị sót không có trong dữ liệu kiểm tra → không ai phát hiện kịp.</t>
+        </is>
+      </c>
       <c r="B16" s="11" t="n"/>
       <c r="C16" s="11" t="n"/>
       <c r="D16" s="11" t="n"/>
@@ -2725,26 +2977,38 @@
       <c r="P16" s="11" t="n"/>
       <c r="Q16" s="11" t="n"/>
       <c r="R16" s="12" t="n"/>
-      <c r="S16" s="11" t="n"/>
-      <c r="T16" s="11" t="n"/>
-      <c r="U16" s="11" t="n"/>
-      <c r="V16" s="11" t="n"/>
-      <c r="W16" s="11" t="n"/>
-      <c r="X16" s="11" t="n"/>
-      <c r="Y16" s="11" t="n"/>
-      <c r="Z16" s="11" t="n"/>
-      <c r="AA16" s="11" t="n"/>
-      <c r="AB16" s="11" t="n"/>
-      <c r="AC16" s="11" t="n"/>
-      <c r="AD16" s="11" t="n"/>
-      <c r="AE16" s="11" t="n"/>
-      <c r="AF16" s="11" t="n"/>
+      <c r="S16" s="163" t="inlineStr">
+        <is>
+          <t>Phát hiện sót / 漏れ検出</t>
+        </is>
+      </c>
+      <c r="T16" s="156" t="n"/>
+      <c r="U16" s="156" t="n"/>
+      <c r="V16" s="157" t="n"/>
+      <c r="W16" s="163" t="inlineStr">
+        <is>
+          <t>Khi hàng không về / 未入荷時</t>
+        </is>
+      </c>
+      <c r="X16" s="156" t="n"/>
+      <c r="Y16" s="156" t="n"/>
+      <c r="Z16" s="157" t="n"/>
+      <c r="AA16" s="155" t="inlineStr">
+        <is>
+          <t>Ngay trong tuần / 週内に検出</t>
+        </is>
+      </c>
+      <c r="AB16" s="156" t="n"/>
+      <c r="AC16" s="156" t="n"/>
+      <c r="AD16" s="156" t="n"/>
+      <c r="AE16" s="156" t="n"/>
+      <c r="AF16" s="157" t="n"/>
       <c r="AG16" s="13" t="n"/>
     </row>
-    <row r="17" ht="16.95" customHeight="1">
-      <c r="A17" s="153" t="inlineStr">
-        <is>
-          <t>【現状 / Hiện trạng】</t>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="167" t="inlineStr">
+        <is>
+          <t>▲ チェックは入荷段階のみ → 発注済みのものしか確認できない。</t>
         </is>
       </c>
       <c r="B17" s="11" t="n"/>
@@ -2763,9 +3027,9 @@
       <c r="O17" s="11" t="n"/>
       <c r="P17" s="11" t="n"/>
       <c r="Q17" s="11" t="n"/>
-      <c r="R17" s="154" t="inlineStr">
-        <is>
-          <t>【改善後 / Sau cải tiến】</t>
+      <c r="R17" s="168" t="inlineStr">
+        <is>
+          <t>▼ File đối chiếu thực tế (Power Query) / 実際の照合ファイル</t>
         </is>
       </c>
       <c r="S17" s="11" t="n"/>
@@ -2784,10 +3048,10 @@
       <c r="AF17" s="11" t="n"/>
       <c r="AG17" s="13" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="148" t="inlineStr">
-        <is>
-          <t>・Tần suất / 照合頻度：Không định kỳ / 不定期</t>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　 発注漏れはデータに存在しないため、誰も気づけない。</t>
         </is>
       </c>
       <c r="B18" s="11" t="n"/>
@@ -2806,11 +3070,7 @@
       <c r="O18" s="11" t="n"/>
       <c r="P18" s="11" t="n"/>
       <c r="Q18" s="11" t="n"/>
-      <c r="R18" s="152" t="inlineStr">
-        <is>
-          <t>・Tần suất / 照合頻度：1 lần/tuần, cố định / 週1回（定期）</t>
-        </is>
-      </c>
+      <c r="R18" s="12" t="n"/>
       <c r="S18" s="11" t="n"/>
       <c r="T18" s="11" t="n"/>
       <c r="U18" s="11" t="n"/>
@@ -2827,12 +3087,8 @@
       <c r="AF18" s="11" t="n"/>
       <c r="AG18" s="13" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="148" t="inlineStr">
-        <is>
-          <t>・Phương thức / 方法：Thủ công bằng Excel / Excel手作業</t>
-        </is>
-      </c>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="10" t="n"/>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
       <c r="D19" s="11" t="n"/>
@@ -2849,11 +3105,7 @@
       <c r="O19" s="11" t="n"/>
       <c r="P19" s="11" t="n"/>
       <c r="Q19" s="11" t="n"/>
-      <c r="R19" s="152" t="inlineStr">
-        <is>
-          <t>・Phương thức / 方法：Tự động, chỉ cần Refresh / 自動（更新のみ）</t>
-        </is>
-      </c>
+      <c r="R19" s="12" t="n"/>
       <c r="S19" s="11" t="n"/>
       <c r="T19" s="11" t="n"/>
       <c r="U19" s="15" t="n"/>
@@ -2870,10 +3122,10 @@
       <c r="AF19" s="11" t="n"/>
       <c r="AG19" s="13" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="148" t="inlineStr">
-        <is>
-          <t>・Phạm vi / 範囲：Kiểm tra từng đơn lẻ / 個別確認のみ</t>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="169" t="inlineStr">
+        <is>
+          <t>Hậu quả khi sót PO / 発注漏れ時の影響</t>
         </is>
       </c>
       <c r="B20" s="11" t="n"/>
@@ -2892,11 +3144,7 @@
       <c r="O20" s="11" t="n"/>
       <c r="P20" s="11" t="n"/>
       <c r="Q20" s="11" t="n"/>
-      <c r="R20" s="152" t="inlineStr">
-        <is>
-          <t>・Phạm vi / 範囲：100% PO / 全PO</t>
-        </is>
-      </c>
+      <c r="R20" s="12" t="n"/>
       <c r="S20" s="11" t="n"/>
       <c r="T20" s="11" t="n"/>
       <c r="U20" s="11" t="n"/>
@@ -2913,10 +3161,10 @@
       <c r="AF20" s="11" t="n"/>
       <c r="AG20" s="13" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="148" t="inlineStr">
-        <is>
-          <t>・Phát hiện sai lệch / 差異検出：Phụ thuộc cá nhân / 担当者任せ</t>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="167" t="inlineStr">
+        <is>
+          <t>① Chỉ lộ ra khi đến ngày cần mà hàng không về / 必要日に未入荷で初めて判明</t>
         </is>
       </c>
       <c r="B21" s="11" t="n"/>
@@ -2935,11 +3183,7 @@
       <c r="O21" s="11" t="n"/>
       <c r="P21" s="11" t="n"/>
       <c r="Q21" s="11" t="n"/>
-      <c r="R21" s="152" t="inlineStr">
-        <is>
-          <t>・Phát hiện sai lệch / 差異検出：Tự động ra danh sách / 自動リスト化</t>
-        </is>
-      </c>
+      <c r="R21" s="12" t="n"/>
       <c r="S21" s="11" t="n"/>
       <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n"/>
@@ -2956,8 +3200,12 @@
       <c r="AF21" s="11" t="n"/>
       <c r="AG21" s="13" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="n"/>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="167" t="inlineStr">
+        <is>
+          <t>② Phải đặt gấp, vận chuyển gấp → tăng chi phí / 緊急発注・特急輸送でコスト増</t>
+        </is>
+      </c>
       <c r="B22" s="11" t="n"/>
       <c r="C22" s="11" t="n"/>
       <c r="D22" s="11" t="n"/>
@@ -2991,8 +3239,12 @@
       <c r="AF22" s="11" t="n"/>
       <c r="AG22" s="13" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="n"/>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="167" t="inlineStr">
+        <is>
+          <t>③ Thiếu linh kiện → chậm lắp ráp, nguy cơ trễ xuất hàng cho khách</t>
+        </is>
+      </c>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="11" t="n"/>
       <c r="D23" s="11" t="n"/>
@@ -3026,8 +3278,12 @@
       <c r="AF23" s="11" t="n"/>
       <c r="AG23" s="13" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="n"/>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　 部品欠品 → 組立遅延・お客様への出荷遅延のリスク</t>
+        </is>
+      </c>
       <c r="B24" s="11" t="n"/>
       <c r="C24" s="11" t="n"/>
       <c r="D24" s="11" t="n"/>
@@ -3061,7 +3317,7 @@
       <c r="AF24" s="17" t="n"/>
       <c r="AG24" s="18" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="17" customHeight="1">
       <c r="A25" s="10" t="n"/>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="11" t="n"/>
@@ -3175,9 +3431,9 @@
       <c r="AG27" s="21" t="n"/>
     </row>
     <row r="28" ht="15" customFormat="1" customHeight="1" s="31">
-      <c r="A28" s="151" t="inlineStr">
-        <is>
-          <t>① Khối lượng công việc lớn → PO phát hành trễ hoặc bị sót.</t>
+      <c r="A28" s="167" t="inlineStr">
+        <is>
+          <t>① Chưa có cơ chế đối chiếu định kỳ giữa Mua hàng và Kế hoạch (mỗi bên 1 file riêng).</t>
         </is>
       </c>
       <c r="B28" s="23" t="n"/>
@@ -3196,9 +3452,9 @@
       <c r="O28" s="23" t="n"/>
       <c r="P28" s="23" t="n"/>
       <c r="Q28" s="24" t="n"/>
-      <c r="R28" s="155" t="inlineStr">
-        <is>
-          <t>① Gần như loại bỏ rủi ro sót PO → sản xuất ổn định hơn.</t>
+      <c r="R28" s="170" t="inlineStr">
+        <is>
+          <t>① Phát hiện sót PO ngay trong tuần, trước khi ảnh hưởng sản xuất → sản xuất ổn định.</t>
         </is>
       </c>
       <c r="S28" s="25" t="n"/>
@@ -3218,9 +3474,9 @@
       <c r="AG28" s="26" t="n"/>
     </row>
     <row r="29" ht="15" customFormat="1" customHeight="1" s="31">
-      <c r="A29" s="156" t="inlineStr">
-        <is>
-          <t>② Theo dõi thủ công bằng Excel → dễ nhầm lẫn, sai sót khi nhập liệu.</t>
+      <c r="A29" s="171" t="inlineStr">
+        <is>
+          <t>② Theo dõi thủ công, phụ thuộc trí nhớ PIC → cao điểm công việc dễ trễ, sót PO.</t>
         </is>
       </c>
       <c r="B29" s="23" t="n"/>
@@ -3239,7 +3495,7 @@
       <c r="O29" s="23" t="n"/>
       <c r="P29" s="23" t="n"/>
       <c r="Q29" s="24" t="n"/>
-      <c r="R29" s="155" t="inlineStr">
+      <c r="R29" s="170" t="inlineStr">
         <is>
           <t>② Số lượng đặt khớp yêu cầu → tránh đặt thừa (tăng chi phí) hoặc thiếu (ảnh hưởng SX).</t>
         </is>
@@ -3264,9 +3520,9 @@
       <c r="AJ29" s="32" t="n"/>
     </row>
     <row r="30" ht="15" customFormat="1" customHeight="1" s="31">
-      <c r="A30" s="156" t="inlineStr">
-        <is>
-          <t>③ PO chưa phát hành → ảnh hưởng kế hoạch lắp ráp và xuất hàng cho khách.</t>
+      <c r="A30" s="171" t="inlineStr">
+        <is>
+          <t>③ Sót PO ảnh hưởng trực tiếp kế hoạch lắp ráp và kế hoạch xuất hàng cho khách.</t>
         </is>
       </c>
       <c r="B30" s="23" t="n"/>
@@ -3285,9 +3541,9 @@
       <c r="O30" s="23" t="n"/>
       <c r="P30" s="23" t="n"/>
       <c r="Q30" s="24" t="n"/>
-      <c r="R30" s="157" t="inlineStr">
-        <is>
-          <t>③ Đối chiếu chuyển từ thủ công sang tự động, chỉ cần Refresh.</t>
+      <c r="R30" s="172" t="inlineStr">
+        <is>
+          <t>③ Đối chiếu chuyển từ thủ công sang tự động, chỉ cần Refresh → giảm tải cho PIC.</t>
         </is>
       </c>
       <c r="S30" s="25" t="n"/>
@@ -3348,9 +3604,9 @@
       <c r="AJ31" s="32" t="n"/>
     </row>
     <row r="32" ht="16.2" customHeight="1">
-      <c r="A32" s="158" t="inlineStr">
-        <is>
-          <t>① 業務量が多い時、POの発行遅れ・漏れが発生する。</t>
+      <c r="A32" s="173" t="inlineStr">
+        <is>
+          <t>① 購買課と計画課の間に定期照合の仕組みがない（各自別ファイル管理）。</t>
         </is>
       </c>
       <c r="B32" s="23" t="n"/>
@@ -3369,9 +3625,9 @@
       <c r="O32" s="23" t="n"/>
       <c r="P32" s="23" t="n"/>
       <c r="Q32" s="24" t="n"/>
-      <c r="R32" s="157" t="inlineStr">
-        <is>
-          <t>① PO漏れリスクをほぼ解消し、生産の安定性が向上。</t>
+      <c r="R32" s="172" t="inlineStr">
+        <is>
+          <t>① 生産に影響する前に、週内でPO漏れを発見 → 生産の安定化。</t>
         </is>
       </c>
       <c r="S32" s="25" t="n"/>
@@ -3394,9 +3650,9 @@
       <c r="AJ32" s="32" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="158" t="inlineStr">
-        <is>
-          <t>② Excel手作業のため、入力ミス・見落としが起きやすい。</t>
+      <c r="A33" s="173" t="inlineStr">
+        <is>
+          <t>② 手作業・担当者の記憶頼み → 業務ピーク時に発行遅れ・漏れが発生。</t>
         </is>
       </c>
       <c r="B33" s="23" t="n"/>
@@ -3415,9 +3671,9 @@
       <c r="O33" s="23" t="n"/>
       <c r="P33" s="23" t="n"/>
       <c r="Q33" s="24" t="n"/>
-      <c r="R33" s="157" t="inlineStr">
-        <is>
-          <t>② 発注数が依頼数と一致し、過剰発注（コスト増）・発注不足を防止。</t>
+      <c r="R33" s="172" t="inlineStr">
+        <is>
+          <t>② 発注数が依頼数と一致 → 過剰発注（コスト増）・発注不足を防止。</t>
         </is>
       </c>
       <c r="S33" s="25" t="n"/>
@@ -3437,9 +3693,9 @@
       <c r="AG33" s="26" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="158" t="inlineStr">
-        <is>
-          <t>③ PO未発行は組立計画・お客様への出荷計画に直接影響する。</t>
+      <c r="A34" s="173" t="inlineStr">
+        <is>
+          <t>③ PO漏れは組立計画・お客様への出荷計画に直接影響する。</t>
         </is>
       </c>
       <c r="B34" s="23" t="n"/>
@@ -3458,9 +3714,9 @@
       <c r="O34" s="23" t="n"/>
       <c r="P34" s="23" t="n"/>
       <c r="Q34" s="24" t="n"/>
-      <c r="R34" s="155" t="inlineStr">
-        <is>
-          <t>③ 照合作業を手作業から自動化、更新のみで完了。</t>
+      <c r="R34" s="170" t="inlineStr">
+        <is>
+          <t>③ 照合作業を手作業から自動化（更新のみ）→ 担当者の負担軽減。</t>
         </is>
       </c>
       <c r="S34" s="25" t="n"/>
@@ -3628,7 +3884,7 @@
       <c r="AG38" s="41" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="151" t="inlineStr">
+      <c r="A39" s="167" t="inlineStr">
         <is>
           <t>Lập file đối chiếu chéo tự động hàng tuần (chi tiết theo sheet đính kèm):</t>
         </is>
@@ -3649,7 +3905,7 @@
       <c r="O39" s="23" t="n"/>
       <c r="P39" s="23" t="n"/>
       <c r="Q39" s="24" t="n"/>
-      <c r="R39" s="149" t="inlineStr">
+      <c r="R39" s="172" t="inlineStr">
         <is>
           <t>① Chuẩn hóa thành quy trình nội bộ: đối chiếu hàng tuần là bước bắt buộc của mỗi PIC.</t>
         </is>
@@ -3671,7 +3927,7 @@
       <c r="AG39" s="42" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="151" t="inlineStr">
+      <c r="A40" s="167" t="inlineStr">
         <is>
           <t>B1: Kết nối dữ liệu Mua hàng và yêu cầu mua của Kế hoạch bằng Power Query.</t>
         </is>
@@ -3692,7 +3948,7 @@
       <c r="O40" s="23" t="n"/>
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="24" t="n"/>
-      <c r="R40" s="155" t="inlineStr">
+      <c r="R40" s="170" t="inlineStr">
         <is>
           <t>② Hình thành thói quen kiểm soát đơn hàng, nâng cao trách nhiệm từng PIC.</t>
         </is>
@@ -3714,7 +3970,7 @@
       <c r="AG40" s="42" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="151" t="inlineStr">
+      <c r="A41" s="167" t="inlineStr">
         <is>
           <t>B2: Refresh hàng tuần → tự động xuất danh sách chênh lệch.</t>
         </is>
@@ -3735,7 +3991,7 @@
       <c r="O41" s="23" t="n"/>
       <c r="P41" s="23" t="n"/>
       <c r="Q41" s="24" t="n"/>
-      <c r="R41" s="149" t="inlineStr">
+      <c r="R41" s="172" t="inlineStr">
         <is>
           <t>③ Nâng cao năng lực cung ứng và uy tín của công ty với khách hàng.</t>
         </is>
@@ -3757,7 +4013,7 @@
       <c r="AG41" s="42" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="151" t="inlineStr">
+      <c r="A42" s="167" t="inlineStr">
         <is>
           <t>B3: Rà soát chênh lệch, xử lý ngay để số lượng PO khớp kế hoạch yêu cầu.</t>
         </is>
@@ -3778,7 +4034,7 @@
       <c r="O42" s="23" t="n"/>
       <c r="P42" s="23" t="n"/>
       <c r="Q42" s="24" t="n"/>
-      <c r="R42" s="159" t="inlineStr">
+      <c r="R42" s="174" t="inlineStr">
         <is>
           <t>④ Có thể mở rộng áp dụng cho bộ phận khác có nghiệp vụ đối chiếu tương tự.</t>
         </is>
@@ -3835,7 +4091,7 @@
       <c r="AG43" s="42" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="151" t="inlineStr">
+      <c r="A44" s="167" t="inlineStr">
         <is>
           <t>週次自動クロスチェックファイルの作成（詳細は添付シート参照）：</t>
         </is>
@@ -3856,7 +4112,7 @@
       <c r="O44" s="23" t="n"/>
       <c r="P44" s="23" t="n"/>
       <c r="Q44" s="24" t="n"/>
-      <c r="R44" s="159" t="inlineStr">
+      <c r="R44" s="174" t="inlineStr">
         <is>
           <t>① 社内手順として標準化し、週次照合を各担当者の必須業務とした。</t>
         </is>
@@ -3878,7 +4134,7 @@
       <c r="AG44" s="42" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="151" t="inlineStr">
+      <c r="A45" s="167" t="inlineStr">
         <is>
           <t>ステップ①：購買の納期実績データと計画課の購入依頼データを</t>
         </is>
@@ -3899,7 +4155,7 @@
       <c r="O45" s="23" t="n"/>
       <c r="P45" s="23" t="n"/>
       <c r="Q45" s="24" t="n"/>
-      <c r="R45" s="159" t="inlineStr">
+      <c r="R45" s="174" t="inlineStr">
         <is>
           <t>② 発注管理の習慣が定着し、各担当者の責任感が向上。</t>
         </is>
@@ -3921,7 +4177,7 @@
       <c r="AG45" s="42" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="151" t="inlineStr">
+      <c r="A46" s="167" t="inlineStr">
         <is>
           <t xml:space="preserve">　　　　　　Power Queryで連携。</t>
         </is>
@@ -3942,7 +4198,7 @@
       <c r="O46" s="23" t="n"/>
       <c r="P46" s="23" t="n"/>
       <c r="Q46" s="24" t="n"/>
-      <c r="R46" s="159" t="inlineStr">
+      <c r="R46" s="174" t="inlineStr">
         <is>
           <t>③ 供給能力の向上、お客様からの信頼向上に貢献。</t>
         </is>
@@ -3964,7 +4220,7 @@
       <c r="AG46" s="42" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="151" t="inlineStr">
+      <c r="A47" s="167" t="inlineStr">
         <is>
           <t>ステップ②：毎週更新し、差異リストを自動抽出。</t>
         </is>
@@ -3985,7 +4241,7 @@
       <c r="O47" s="23" t="n"/>
       <c r="P47" s="23" t="n"/>
       <c r="Q47" s="24" t="n"/>
-      <c r="R47" s="159" t="inlineStr">
+      <c r="R47" s="174" t="inlineStr">
         <is>
           <t>④ 同様の照合業務がある他部署へ横展開が可能。</t>
         </is>
@@ -4007,7 +4263,7 @@
       <c r="AG47" s="42" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="151" t="inlineStr">
+      <c r="A48" s="167" t="inlineStr">
         <is>
           <t>ステップ③：差異を確認し、PO数量を依頼計画と一致させる。</t>
         </is>
@@ -4081,24 +4337,47 @@
       <c r="AG49" s="47" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="36">
     <mergeCell ref="V5:X7"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="AA15:AF15"/>
+    <mergeCell ref="Y5:AA7"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="G12:K14"/>
+    <mergeCell ref="W14:Z14"/>
+    <mergeCell ref="AA16:AF16"/>
     <mergeCell ref="AC3:AG3"/>
+    <mergeCell ref="W13:Z13"/>
+    <mergeCell ref="S16:V16"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="Y3:AB3"/>
+    <mergeCell ref="S12:V12"/>
+    <mergeCell ref="A2:J3"/>
+    <mergeCell ref="W15:Z15"/>
+    <mergeCell ref="AA12:AF12"/>
     <mergeCell ref="A6:F7"/>
-    <mergeCell ref="Y5:AA7"/>
-    <mergeCell ref="AB5:AD7"/>
     <mergeCell ref="G5:U7"/>
     <mergeCell ref="AE5:AG7"/>
+    <mergeCell ref="AA14:AF14"/>
+    <mergeCell ref="Y4:AA4"/>
+    <mergeCell ref="AE4:AG4"/>
+    <mergeCell ref="S14:V14"/>
+    <mergeCell ref="AB5:AD7"/>
+    <mergeCell ref="N12:Q14"/>
+    <mergeCell ref="S13:V13"/>
+    <mergeCell ref="AA13:AF13"/>
+    <mergeCell ref="W16:Z16"/>
     <mergeCell ref="V4:X4"/>
-    <mergeCell ref="Y3:AB3"/>
-    <mergeCell ref="Y4:AA4"/>
     <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="B12:D14"/>
     <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A2:J3"/>
-    <mergeCell ref="AE4:AG4"/>
+    <mergeCell ref="W12:Z12"/>
+    <mergeCell ref="S15:V15"/>
   </mergeCells>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.196850393700787" right="0.16" top="0.16" bottom="0" header="0.16" footer="0.16"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="69"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>